<commit_message>
Synchronize operational scenarios and verify all dashboard selectors
</commit_message>
<xml_diff>
--- a/entregas/EFCC_Final/Parametros_Ativos_EFCC.xlsx
+++ b/entregas/EFCC_Final/Parametros_Ativos_EFCC.xlsx
@@ -212,13 +212,13 @@
     <t>DASH 05 V06!N23</t>
   </si>
   <si>
-    <t>ADR Custom</t>
+    <t>ADR · apenas Custom</t>
   </si>
   <si>
     <t>DASH 05 V06!H25</t>
   </si>
   <si>
-    <t>Ocupação Custom</t>
+    <t>Ocupação · apenas Custom</t>
   </si>
   <si>
     <t>DASH 05 V06!H27</t>

</xml_diff>